<commit_message>
Update course plans and educational program documents with quality note revisions and corrections
- TR1034.md: Updated quality notes from 5 to 4; corrected spelling and formatting issues.
- TR2004.md: Updated quality notes from 8 to 7; corrected spelling and formatting issues.
- TR3006.md: Updated quality notes from 6 to 4; corrected spelling and formatting issues.
- AS2002.md: Updated quality notes from 6 to 5; corrected spelling and formatting issues.
- AS3002.md: Updated quality notes from 8 to 7; corrected spelling and formatting issues.
- AS3009.md: Updated quality notes from 6 to 5; corrected spelling and formatting issues.
- AS3012.md: Updated quality notes from 6 to 5; corrected spelling and formatting issues.
- AS4003.md: Updated quality notes from 7 to 6; corrected spelling and formatting issues.
- SENGR.md: Updated quality notes from 7 to 5; corrected spelling and formatting issues.
- Updated multiple Excel files related to grading and assessments.
</commit_message>
<xml_diff>
--- a/vault-dalarna-university/03 IKS/Analys/Betygsrapportering.xlsx
+++ b/vault-dalarna-university/03 IKS/Analys/Betygsrapportering.xlsx
@@ -14403,7 +14403,7 @@
       </c>
       <c r="F412" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F. Aktivt deltagande i seminarierna G/U Slutbetyget på kursen sätts efter en samlad bedömning …</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F. Aktivt deltagande i seminarierna G/U…</t>
         </is>
       </c>
       <c r="G412" s="2" t="inlineStr">
@@ -15961,7 +15961,7 @@
       </c>
       <c r="F458" t="inlineStr">
         <is>
-          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F. Betygsrapportering: Moment 1: Vetenskapsteori - 8 hp Moment 2: Metod - 8 hp…</t>
+          <t>Betyg skrivet utan punktlista: Som betygsskala används A–F. Betygsrapportering:…</t>
         </is>
       </c>
       <c r="G458" s="2" t="inlineStr">

</xml_diff>